<commit_message>
feat: refactor ERP - them module don hang, hoa don, cong no, bao cao va kho
- Them module: orders, invoices, loans, reports, warehouse (stock in/out, tickets), targets, deposits, expenses, revenue, units, positions, price-list, promotions, shipping-fees, partner-units
- Bo cac man hinh cu: delivery, dvgt, kpi, sales, branchloans
- Bo sung test API va excel nhap lieu mau
- Cap nhat docs va cau hinh electron-builder

Co-authored-by: CommandCodeBot <noreply@commandcode.ai>
</commit_message>
<xml_diff>
--- a/excel/Nước thương mại.xlsx
+++ b/excel/Nước thương mại.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Agentic-AI\Doing\QLBanHang-main\QLBanHang\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC1E2F9E-9325-4A8E-B6EE-DB9DE60FF774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AED9A86B-781E-4C4E-AEA2-77107991067B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -263,47 +263,17 @@
   </cellStyleXfs>
   <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -334,6 +304,36 @@
     </xf>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -651,847 +651,861 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="9" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
-      <c r="M1" s="9"/>
-      <c r="N1" s="9"/>
-      <c r="O1" s="9"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
+      <c r="N1" s="17"/>
+      <c r="O1" s="17"/>
     </row>
     <row r="2" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="8" t="s">
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
-      <c r="L2" s="8"/>
-      <c r="M2" s="8"/>
-      <c r="N2" s="8"/>
-      <c r="O2" s="8"/>
+      <c r="I2" s="25"/>
+      <c r="J2" s="25"/>
+      <c r="K2" s="25"/>
+      <c r="L2" s="25"/>
+      <c r="M2" s="25"/>
+      <c r="N2" s="25"/>
+      <c r="O2" s="25"/>
     </row>
     <row r="4" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
-      <c r="L4" s="7"/>
-      <c r="M4" s="7"/>
-      <c r="N4" s="7"/>
-      <c r="O4" s="7"/>
+      <c r="B4" s="26"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="26"/>
+      <c r="K4" s="26"/>
+      <c r="L4" s="26"/>
+      <c r="M4" s="26"/>
+      <c r="N4" s="26"/>
+      <c r="O4" s="26"/>
     </row>
     <row r="5" spans="1:16" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
-      <c r="M5" s="6"/>
-      <c r="N5" s="6"/>
-      <c r="O5" s="6"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="21"/>
+      <c r="I5" s="21"/>
+      <c r="J5" s="21"/>
+      <c r="K5" s="21"/>
+      <c r="L5" s="21"/>
+      <c r="M5" s="21"/>
+      <c r="N5" s="21"/>
+      <c r="O5" s="21"/>
     </row>
     <row r="6" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="13"/>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13">
+      <c r="A6" s="5"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5">
         <v>78704</v>
       </c>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13">
+      <c r="D6" s="5"/>
+      <c r="E6" s="5">
         <v>86111</v>
       </c>
-      <c r="F6" s="13"/>
-      <c r="G6" s="13">
+      <c r="F6" s="5"/>
+      <c r="G6" s="5">
         <v>90741</v>
       </c>
-      <c r="H6" s="13"/>
-      <c r="I6" s="13">
+      <c r="H6" s="5"/>
+      <c r="I6" s="5">
         <v>98149</v>
       </c>
-      <c r="J6" s="13"/>
-      <c r="K6" s="13">
+      <c r="J6" s="5"/>
+      <c r="K6" s="5">
         <v>48148</v>
       </c>
-      <c r="L6" s="13"/>
-      <c r="M6" s="13">
+      <c r="L6" s="5"/>
+      <c r="M6" s="5">
         <v>44444</v>
       </c>
-      <c r="N6" s="13"/>
-      <c r="O6" s="13"/>
+      <c r="N6" s="5"/>
+      <c r="O6" s="5"/>
     </row>
     <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4" t="s">
+      <c r="C7" s="23"/>
+      <c r="D7" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4" t="s">
+      <c r="E7" s="23"/>
+      <c r="F7" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4" t="s">
+      <c r="G7" s="23"/>
+      <c r="H7" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4" t="s">
+      <c r="I7" s="23"/>
+      <c r="J7" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4" t="s">
+      <c r="K7" s="23"/>
+      <c r="L7" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="M7" s="4"/>
-      <c r="N7" s="4" t="s">
+      <c r="M7" s="23"/>
+      <c r="N7" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="O7" s="4"/>
-      <c r="P7" s="3"/>
+      <c r="O7" s="23"/>
+      <c r="P7" s="18"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A8" s="5"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
-      <c r="M8" s="4"/>
-      <c r="N8" s="4"/>
-      <c r="O8" s="4"/>
-      <c r="P8" s="3"/>
+      <c r="A8" s="22"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="23"/>
+      <c r="I8" s="23"/>
+      <c r="J8" s="23"/>
+      <c r="K8" s="23"/>
+      <c r="L8" s="23"/>
+      <c r="M8" s="23"/>
+      <c r="N8" s="23"/>
+      <c r="O8" s="23"/>
+      <c r="P8" s="18"/>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A9" s="5"/>
-      <c r="B9" s="14" t="s">
+      <c r="A9" s="22"/>
+      <c r="B9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="D9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="F9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G9" s="14" t="s">
+      <c r="G9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H9" s="14" t="s">
+      <c r="H9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="I9" s="14" t="s">
+      <c r="I9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J9" s="14" t="s">
+      <c r="J9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="K9" s="14" t="s">
+      <c r="K9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="L9" s="14" t="s">
+      <c r="L9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="M9" s="14" t="s">
+      <c r="M9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="N9" s="14" t="s">
+      <c r="N9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="O9" s="14" t="s">
+      <c r="O9" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
-      <c r="N10" s="2"/>
-      <c r="O10" s="2"/>
+      <c r="B10" s="19"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="19"/>
+      <c r="I10" s="19"/>
+      <c r="J10" s="19"/>
+      <c r="K10" s="19"/>
+      <c r="L10" s="19"/>
+      <c r="M10" s="19"/>
+      <c r="N10" s="19"/>
+      <c r="O10" s="19"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A11" s="16" t="s">
+      <c r="A11" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="17">
+      <c r="B11" s="7">
         <v>401</v>
       </c>
-      <c r="C11" s="18">
+      <c r="C11" s="8">
         <f>B11*C6</f>
         <v>31560304</v>
       </c>
-      <c r="D11" s="18">
+      <c r="D11" s="8">
         <v>0</v>
       </c>
-      <c r="E11" s="18">
+      <c r="E11" s="8">
         <v>0</v>
       </c>
-      <c r="F11" s="18">
+      <c r="F11" s="8">
         <v>2082</v>
       </c>
-      <c r="G11" s="18">
+      <c r="G11" s="8">
         <f>F11*G6</f>
         <v>188922762</v>
       </c>
-      <c r="H11" s="18">
+      <c r="H11" s="8">
         <v>5</v>
       </c>
-      <c r="I11" s="18">
+      <c r="I11" s="8">
         <f>H11*I6</f>
         <v>490745</v>
       </c>
-      <c r="J11" s="18">
+      <c r="J11" s="8">
         <v>103</v>
       </c>
-      <c r="K11" s="18">
+      <c r="K11" s="8">
         <f>J11*K6</f>
         <v>4959244</v>
       </c>
-      <c r="L11" s="18">
+      <c r="L11" s="8">
         <v>133</v>
       </c>
-      <c r="M11" s="18">
+      <c r="M11" s="8">
         <f>L11*M6</f>
         <v>5911052</v>
       </c>
-      <c r="N11" s="18">
+      <c r="N11" s="8">
         <f>B11+D11+F11+H11+J11+L11</f>
         <v>2724</v>
       </c>
-      <c r="O11" s="18">
+      <c r="O11" s="8">
         <f>C11+E11+G11+I11+K11+M11</f>
         <v>231844107</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="20">
+      <c r="B12" s="10">
         <v>401</v>
       </c>
-      <c r="C12" s="18">
+      <c r="C12" s="8">
         <v>31560304</v>
       </c>
-      <c r="D12" s="21">
+      <c r="D12" s="11">
         <v>0</v>
       </c>
-      <c r="E12" s="21">
+      <c r="E12" s="11">
         <v>0</v>
       </c>
-      <c r="F12" s="21">
+      <c r="F12" s="11">
         <v>2082</v>
       </c>
-      <c r="G12" s="21">
+      <c r="G12" s="11">
         <v>188922762</v>
       </c>
-      <c r="H12" s="21">
+      <c r="H12" s="11">
         <v>5</v>
       </c>
-      <c r="I12" s="21">
+      <c r="I12" s="11">
         <v>490745</v>
       </c>
-      <c r="J12" s="21">
+      <c r="J12" s="11">
         <v>103</v>
       </c>
-      <c r="K12" s="21">
+      <c r="K12" s="11">
         <v>4959244</v>
       </c>
-      <c r="L12" s="21">
+      <c r="L12" s="11">
         <v>133</v>
       </c>
-      <c r="M12" s="21">
+      <c r="M12" s="11">
         <v>5911052</v>
       </c>
-      <c r="N12" s="21">
+      <c r="N12" s="11">
         <f>B12+D12+F12+H12+J12+L12</f>
         <v>2724</v>
       </c>
-      <c r="O12" s="21">
+      <c r="O12" s="11">
         <f>C12+E12+G12+I12+K12+M12</f>
         <v>231844107</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
-      <c r="N13" s="2"/>
-      <c r="O13" s="2"/>
+      <c r="B13" s="19"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="19"/>
+      <c r="I13" s="19"/>
+      <c r="J13" s="19"/>
+      <c r="K13" s="19"/>
+      <c r="L13" s="19"/>
+      <c r="M13" s="19"/>
+      <c r="N13" s="19"/>
+      <c r="O13" s="19"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="17">
-        <f t="shared" ref="B14:O14" si="0">B12+B30</f>
+      <c r="B14" s="7">
+        <f>B12+B30</f>
         <v>1053</v>
       </c>
-      <c r="C14" s="18">
-        <f t="shared" si="0"/>
+      <c r="C14" s="8">
+        <f>C12+C30</f>
         <v>82875312</v>
       </c>
-      <c r="D14" s="18">
-        <f t="shared" si="0"/>
+      <c r="D14" s="8">
+        <f>D12+D30</f>
         <v>89</v>
       </c>
-      <c r="E14" s="18">
-        <f t="shared" si="0"/>
+      <c r="E14" s="8">
+        <f>E12+E30</f>
         <v>7663879</v>
       </c>
-      <c r="F14" s="18">
-        <f t="shared" si="0"/>
+      <c r="F14" s="8">
+        <f>F12+F30</f>
         <v>9236</v>
       </c>
-      <c r="G14" s="18">
-        <f t="shared" si="0"/>
+      <c r="G14" s="8">
+        <f>G12+G30</f>
         <v>838083876</v>
       </c>
-      <c r="H14" s="18">
-        <f t="shared" si="0"/>
+      <c r="H14" s="8">
+        <f>H12+H30</f>
         <v>289</v>
       </c>
-      <c r="I14" s="18">
-        <f t="shared" si="0"/>
+      <c r="I14" s="8">
+        <f>I12+I30</f>
         <v>28365061</v>
       </c>
-      <c r="J14" s="18">
-        <f t="shared" si="0"/>
+      <c r="J14" s="8">
+        <f>J12+J30</f>
         <v>393</v>
       </c>
-      <c r="K14" s="18">
-        <f t="shared" si="0"/>
+      <c r="K14" s="8">
+        <f>K12+K30</f>
         <v>18922164</v>
       </c>
-      <c r="L14" s="18">
-        <f t="shared" si="0"/>
+      <c r="L14" s="8">
+        <f>L12+L30</f>
         <v>474</v>
       </c>
-      <c r="M14" s="18">
-        <f t="shared" si="0"/>
+      <c r="M14" s="8">
+        <f>M12+M30</f>
         <v>21066456</v>
       </c>
-      <c r="N14" s="18">
-        <f t="shared" si="0"/>
+      <c r="N14" s="8">
+        <f>N12+N30</f>
         <v>11534</v>
       </c>
-      <c r="O14" s="18">
-        <f t="shared" si="0"/>
+      <c r="O14" s="8">
+        <f>O12+O30</f>
         <v>996976748</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="20">
+      <c r="B15" s="10">
         <v>652</v>
       </c>
-      <c r="C15" s="18">
+      <c r="C15" s="8">
         <v>51315008</v>
       </c>
-      <c r="D15" s="21">
+      <c r="D15" s="11">
         <v>89</v>
       </c>
-      <c r="E15" s="21">
+      <c r="E15" s="11">
         <v>7663879</v>
       </c>
-      <c r="F15" s="21">
+      <c r="F15" s="11">
         <v>7154</v>
       </c>
-      <c r="G15" s="21">
+      <c r="G15" s="11">
         <v>649161114</v>
       </c>
-      <c r="H15" s="21">
+      <c r="H15" s="11">
         <v>284</v>
       </c>
-      <c r="I15" s="21">
+      <c r="I15" s="11">
         <v>27874316</v>
       </c>
-      <c r="J15" s="21">
+      <c r="J15" s="11">
         <v>290</v>
       </c>
-      <c r="K15" s="21">
+      <c r="K15" s="11">
         <v>13962920</v>
       </c>
-      <c r="L15" s="21">
+      <c r="L15" s="11">
         <v>341</v>
       </c>
-      <c r="M15" s="21">
+      <c r="M15" s="11">
         <v>15155404</v>
       </c>
-      <c r="N15" s="21">
+      <c r="N15" s="11">
         <v>8810</v>
       </c>
-      <c r="O15" s="21">
+      <c r="O15" s="11">
         <v>765132641</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="11"/>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="11"/>
-      <c r="J16" s="11"/>
-      <c r="K16" s="11"/>
-      <c r="L16" s="11"/>
-      <c r="M16" s="11"/>
-      <c r="N16" s="11"/>
-      <c r="O16" s="11"/>
+      <c r="A16" s="3"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
+      <c r="L16" s="3"/>
+      <c r="M16" s="3"/>
+      <c r="N16" s="3"/>
+      <c r="O16" s="3"/>
     </row>
     <row r="17" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="1" t="s">
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="11"/>
-      <c r="K17" s="11"/>
-      <c r="L17" s="1" t="s">
+      <c r="G17" s="20"/>
+      <c r="H17" s="20"/>
+      <c r="I17" s="20"/>
+      <c r="J17" s="3"/>
+      <c r="K17" s="3"/>
+      <c r="L17" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="M17" s="1"/>
-      <c r="N17" s="1"/>
-      <c r="O17" s="1"/>
+      <c r="M17" s="20"/>
+      <c r="N17" s="20"/>
+      <c r="O17" s="20"/>
     </row>
     <row r="18" spans="1:15" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A18" s="22"/>
-      <c r="B18" s="22"/>
-      <c r="C18" s="22"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="22"/>
-      <c r="I18" s="22"/>
-      <c r="J18" s="22"/>
-      <c r="K18" s="22"/>
-      <c r="L18" s="22"/>
-      <c r="M18" s="22"/>
-      <c r="N18" s="22"/>
-      <c r="O18" s="22"/>
+      <c r="A18" s="12"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="12"/>
+      <c r="K18" s="12"/>
+      <c r="L18" s="12"/>
+      <c r="M18" s="12"/>
+      <c r="N18" s="12"/>
+      <c r="O18" s="12"/>
     </row>
     <row r="19" spans="1:15" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A19" s="22"/>
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="22"/>
-      <c r="H19" s="22"/>
-      <c r="I19" s="22"/>
-      <c r="J19" s="22"/>
-      <c r="K19" s="22"/>
-      <c r="L19" s="22"/>
-      <c r="M19" s="22"/>
-      <c r="N19" s="22"/>
-      <c r="O19" s="22"/>
+      <c r="A19" s="12"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="12"/>
+      <c r="K19" s="12"/>
+      <c r="L19" s="12"/>
+      <c r="M19" s="12"/>
+      <c r="N19" s="12"/>
+      <c r="O19" s="12"/>
     </row>
     <row r="20" spans="1:15" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A20" s="22"/>
-      <c r="B20" s="22"/>
-      <c r="C20" s="22"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="22"/>
-      <c r="H20" s="22"/>
-      <c r="I20" s="22"/>
-      <c r="J20" s="22"/>
-      <c r="K20" s="22"/>
-      <c r="L20" s="22"/>
-      <c r="M20" s="22"/>
-      <c r="N20" s="22"/>
-      <c r="O20" s="22"/>
+      <c r="A20" s="12"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="12"/>
+      <c r="I20" s="12"/>
+      <c r="J20" s="12"/>
+      <c r="K20" s="12"/>
+      <c r="L20" s="12"/>
+      <c r="M20" s="12"/>
+      <c r="N20" s="12"/>
+      <c r="O20" s="12"/>
     </row>
     <row r="22" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="9" t="s">
+      <c r="A22" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="B22" s="9"/>
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="23"/>
-      <c r="F22" s="9" t="s">
+      <c r="B22" s="17"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="G22" s="9"/>
-      <c r="H22" s="9"/>
-      <c r="I22" s="9"/>
-      <c r="J22" s="23"/>
-      <c r="K22" s="23"/>
-      <c r="L22" s="9" t="s">
+      <c r="G22" s="17"/>
+      <c r="H22" s="17"/>
+      <c r="I22" s="17"/>
+      <c r="J22" s="13"/>
+      <c r="K22" s="13"/>
+      <c r="L22" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="M22" s="9"/>
-      <c r="N22" s="9"/>
-      <c r="O22" s="9"/>
+      <c r="M22" s="17"/>
+      <c r="N22" s="17"/>
+      <c r="O22" s="17"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A26" s="16" t="s">
+      <c r="A26" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B26" s="17">
+      <c r="B26" s="7">
         <v>63</v>
       </c>
-      <c r="C26" s="18">
+      <c r="C26" s="8">
         <v>4958352</v>
       </c>
-      <c r="D26" s="18">
+      <c r="D26" s="8">
         <v>0</v>
       </c>
-      <c r="E26" s="18">
+      <c r="E26" s="8">
         <v>0</v>
       </c>
-      <c r="F26" s="18">
+      <c r="F26" s="8">
         <v>982</v>
       </c>
-      <c r="G26" s="18">
+      <c r="G26" s="8">
         <v>89107662</v>
       </c>
-      <c r="H26" s="18">
+      <c r="H26" s="8">
         <v>20</v>
       </c>
-      <c r="I26" s="18">
+      <c r="I26" s="8">
         <v>1962980</v>
       </c>
-      <c r="J26" s="18">
+      <c r="J26" s="8">
         <v>36</v>
       </c>
-      <c r="K26" s="18">
+      <c r="K26" s="8">
         <v>1733328</v>
       </c>
-      <c r="L26" s="18">
+      <c r="L26" s="8">
         <v>61</v>
       </c>
-      <c r="M26" s="18">
+      <c r="M26" s="8">
         <v>2711084</v>
       </c>
-      <c r="N26" s="18">
+      <c r="N26" s="8">
         <v>1162</v>
       </c>
-      <c r="O26" s="18">
+      <c r="O26" s="8">
         <v>100473406</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A27" s="19" t="s">
+      <c r="A27" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B27" s="20">
+      <c r="B27" s="10">
         <v>63</v>
       </c>
-      <c r="C27" s="21">
+      <c r="C27" s="11">
         <v>4958352</v>
       </c>
-      <c r="D27" s="21">
+      <c r="D27" s="11">
         <v>0</v>
       </c>
-      <c r="E27" s="21">
+      <c r="E27" s="11">
         <v>0</v>
       </c>
-      <c r="F27" s="21">
+      <c r="F27" s="11">
         <v>982</v>
       </c>
-      <c r="G27" s="21">
+      <c r="G27" s="11">
         <v>89107662</v>
       </c>
-      <c r="H27" s="21">
+      <c r="H27" s="11">
         <v>20</v>
       </c>
-      <c r="I27" s="21">
+      <c r="I27" s="11">
         <v>1962980</v>
       </c>
-      <c r="J27" s="21">
+      <c r="J27" s="11">
         <v>36</v>
       </c>
-      <c r="K27" s="21">
+      <c r="K27" s="11">
         <v>1733328</v>
       </c>
-      <c r="L27" s="21">
+      <c r="L27" s="11">
         <v>61</v>
       </c>
-      <c r="M27" s="21">
+      <c r="M27" s="11">
         <v>2711084</v>
       </c>
-      <c r="N27" s="21">
+      <c r="N27" s="11">
         <v>1162</v>
       </c>
-      <c r="O27" s="21">
+      <c r="O27" s="11">
         <v>100473406</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A28" s="15" t="s">
+      <c r="A28" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B28" s="15"/>
-      <c r="C28" s="15"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="15"/>
-      <c r="F28" s="15"/>
-      <c r="G28" s="15"/>
-      <c r="H28" s="15"/>
-      <c r="I28" s="15"/>
-      <c r="J28" s="15"/>
-      <c r="K28" s="15"/>
-      <c r="L28" s="15"/>
-      <c r="M28" s="15"/>
-      <c r="N28" s="15"/>
-      <c r="O28" s="15"/>
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+      <c r="K28" s="1"/>
+      <c r="L28" s="1"/>
+      <c r="M28" s="1"/>
+      <c r="N28" s="1"/>
+      <c r="O28" s="1"/>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A29" s="16" t="s">
+      <c r="A29" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B29" s="17">
+      <c r="B29" s="7">
         <v>126</v>
       </c>
-      <c r="C29" s="18">
+      <c r="C29" s="8">
         <v>4958352</v>
       </c>
-      <c r="D29" s="18">
+      <c r="D29" s="8">
         <v>0</v>
       </c>
-      <c r="E29" s="18">
+      <c r="E29" s="8">
         <v>0</v>
       </c>
-      <c r="F29" s="18">
+      <c r="F29" s="8">
         <v>1964</v>
       </c>
-      <c r="G29" s="18">
+      <c r="G29" s="8">
         <v>89107662</v>
       </c>
-      <c r="H29" s="18">
+      <c r="H29" s="8">
         <v>40</v>
       </c>
-      <c r="I29" s="18">
+      <c r="I29" s="8">
         <v>1962980</v>
       </c>
-      <c r="J29" s="18">
+      <c r="J29" s="8">
         <v>72</v>
       </c>
-      <c r="K29" s="18">
+      <c r="K29" s="8">
         <v>1733328</v>
       </c>
-      <c r="L29" s="18">
+      <c r="L29" s="8">
         <v>122</v>
       </c>
-      <c r="M29" s="18">
+      <c r="M29" s="8">
         <v>2711084</v>
       </c>
-      <c r="N29" s="18">
+      <c r="N29" s="8">
         <v>2324</v>
       </c>
-      <c r="O29" s="18">
+      <c r="O29" s="8">
         <v>100473406</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A30" s="19" t="s">
+      <c r="A30" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B30" s="20">
+      <c r="B30" s="10">
         <v>652</v>
       </c>
-      <c r="C30" s="21">
+      <c r="C30" s="11">
         <v>51315008</v>
       </c>
-      <c r="D30" s="21">
+      <c r="D30" s="11">
         <v>89</v>
       </c>
-      <c r="E30" s="21">
+      <c r="E30" s="11">
         <v>7663879</v>
       </c>
-      <c r="F30" s="21">
+      <c r="F30" s="11">
         <v>7154</v>
       </c>
-      <c r="G30" s="21">
+      <c r="G30" s="11">
         <v>649161114</v>
       </c>
-      <c r="H30" s="21">
+      <c r="H30" s="11">
         <v>284</v>
       </c>
-      <c r="I30" s="21">
+      <c r="I30" s="11">
         <v>27874316</v>
       </c>
-      <c r="J30" s="21">
+      <c r="J30" s="11">
         <v>290</v>
       </c>
-      <c r="K30" s="21">
+      <c r="K30" s="11">
         <v>13962920</v>
       </c>
-      <c r="L30" s="21">
+      <c r="L30" s="11">
         <v>341</v>
       </c>
-      <c r="M30" s="21">
+      <c r="M30" s="11">
         <v>15155404</v>
       </c>
-      <c r="N30" s="21">
+      <c r="N30" s="11">
         <v>8810</v>
       </c>
-      <c r="O30" s="21">
+      <c r="O30" s="11">
         <v>765132641</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="B31" s="24"/>
-      <c r="C31" s="18"/>
-      <c r="D31" s="18"/>
-      <c r="E31" s="18"/>
-      <c r="F31" s="18"/>
-      <c r="G31" s="18"/>
-      <c r="H31" s="18"/>
-      <c r="I31" s="18"/>
-      <c r="J31" s="18"/>
-      <c r="K31" s="18"/>
-      <c r="L31" s="18"/>
-      <c r="M31" s="18"/>
-      <c r="N31" s="18"/>
-      <c r="O31" s="18"/>
+      <c r="B31" s="14"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="8"/>
+      <c r="F31" s="8"/>
+      <c r="G31" s="8"/>
+      <c r="H31" s="8"/>
+      <c r="I31" s="8"/>
+      <c r="J31" s="8"/>
+      <c r="K31" s="8"/>
+      <c r="L31" s="8"/>
+      <c r="M31" s="8"/>
+      <c r="N31" s="8"/>
+      <c r="O31" s="8"/>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="B32" s="25"/>
-      <c r="C32" s="21"/>
-      <c r="D32" s="21"/>
-      <c r="E32" s="21"/>
-      <c r="F32" s="21"/>
-      <c r="G32" s="21"/>
-      <c r="H32" s="21"/>
-      <c r="I32" s="21"/>
-      <c r="J32" s="21"/>
-      <c r="K32" s="21"/>
-      <c r="L32" s="21"/>
-      <c r="M32" s="21"/>
-      <c r="N32" s="21"/>
-      <c r="O32" s="21"/>
+      <c r="B32" s="15"/>
+      <c r="C32" s="11"/>
+      <c r="D32" s="11"/>
+      <c r="E32" s="11"/>
+      <c r="F32" s="11"/>
+      <c r="G32" s="11"/>
+      <c r="H32" s="11"/>
+      <c r="I32" s="11"/>
+      <c r="J32" s="11"/>
+      <c r="K32" s="11"/>
+      <c r="L32" s="11"/>
+      <c r="M32" s="11"/>
+      <c r="N32" s="11"/>
+      <c r="O32" s="11"/>
     </row>
     <row r="33" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B33" s="25"/>
-      <c r="C33" s="25"/>
-      <c r="D33" s="25"/>
-      <c r="E33" s="25"/>
-      <c r="F33" s="25"/>
-      <c r="G33" s="25"/>
-      <c r="H33" s="25"/>
-      <c r="I33" s="25"/>
-      <c r="J33" s="25"/>
-      <c r="K33" s="25"/>
-      <c r="L33" s="25"/>
-      <c r="M33" s="25"/>
-      <c r="N33" s="25"/>
-      <c r="O33" s="25"/>
+      <c r="B33" s="15"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="15"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="15"/>
+      <c r="H33" s="15"/>
+      <c r="I33" s="15"/>
+      <c r="J33" s="15"/>
+      <c r="K33" s="15"/>
+      <c r="L33" s="15"/>
+      <c r="M33" s="15"/>
+      <c r="N33" s="15"/>
+      <c r="O33" s="15"/>
     </row>
     <row r="34" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B34" s="25"/>
-      <c r="C34" s="26"/>
-      <c r="D34" s="26"/>
-      <c r="E34" s="26"/>
-      <c r="F34" s="26"/>
-      <c r="G34" s="26"/>
-      <c r="H34" s="26"/>
-      <c r="I34" s="26"/>
-      <c r="J34" s="26"/>
-      <c r="K34" s="26"/>
-      <c r="L34" s="26"/>
-      <c r="M34" s="26"/>
-      <c r="N34" s="26"/>
-      <c r="O34" s="26"/>
+      <c r="B34" s="15"/>
+      <c r="C34" s="16"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="16"/>
+      <c r="F34" s="16"/>
+      <c r="G34" s="16"/>
+      <c r="H34" s="16"/>
+      <c r="I34" s="16"/>
+      <c r="J34" s="16"/>
+      <c r="K34" s="16"/>
+      <c r="L34" s="16"/>
+      <c r="M34" s="16"/>
+      <c r="N34" s="16"/>
+      <c r="O34" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="H1:O1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="H2:O2"/>
+    <mergeCell ref="A4:O4"/>
+    <mergeCell ref="A5:O5"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="B7:C8"/>
+    <mergeCell ref="D7:E8"/>
+    <mergeCell ref="F7:G8"/>
+    <mergeCell ref="H7:I8"/>
+    <mergeCell ref="J7:K8"/>
+    <mergeCell ref="L7:M8"/>
+    <mergeCell ref="N7:O8"/>
     <mergeCell ref="A22:D22"/>
     <mergeCell ref="F22:I22"/>
     <mergeCell ref="L22:O22"/>
@@ -1501,20 +1515,6 @@
     <mergeCell ref="A17:D17"/>
     <mergeCell ref="F17:I17"/>
     <mergeCell ref="L17:O17"/>
-    <mergeCell ref="A5:O5"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="B7:C8"/>
-    <mergeCell ref="D7:E8"/>
-    <mergeCell ref="F7:G8"/>
-    <mergeCell ref="H7:I8"/>
-    <mergeCell ref="J7:K8"/>
-    <mergeCell ref="L7:M8"/>
-    <mergeCell ref="N7:O8"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="H1:O1"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="H2:O2"/>
-    <mergeCell ref="A4:O4"/>
   </mergeCells>
   <pageMargins left="0.29027777777777802" right="0.17013888888888901" top="0.25972222222222202" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>